<commit_message>
Work on Excel file upload, api routes and much more
</commit_message>
<xml_diff>
--- a/documents/SADV collections upload template.xlsx
+++ b/documents/SADV collections upload template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darryllrobinson/Documents/projects/ciab/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EDA3C8-C60E-CF45-87A5-96DA70EEED7B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0975CFEB-6649-7D49-AEAB-8A7BA895D83D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="960" windowWidth="27640" windowHeight="16000" xr2:uid="{B1A7F133-870B-BE4E-A664-D1E75F837A44}"/>
   </bookViews>
@@ -98,15 +98,9 @@
     <t>arg</t>
   </si>
   <si>
-    <t>dateCreated</t>
-  </si>
-  <si>
     <t>createdBy</t>
   </si>
   <si>
-    <t>f_customerId</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
@@ -117,6 +111,12 @@
   </si>
   <si>
     <t>telephone</t>
+  </si>
+  <si>
+    <t>customerRefNo</t>
+  </si>
+  <si>
+    <t>representativeName</t>
   </si>
 </sst>
 </file>
@@ -470,6 +470,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264374CA-EBDB-1348-8948-C7AE36E6EA27}">
   <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3.83203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12" customWidth="1"/>
+    <col min="24" max="24" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -539,22 +564,22 @@
         <v>21</v>
       </c>
       <c r="W1" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" t="s">
         <v>25</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>